<commit_message>
add sheet festure for validastion
</commit_message>
<xml_diff>
--- a/Duplicate_Payroll_Test_File_Feb26.xlsx
+++ b/Duplicate_Payroll_Test_File_Feb26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\firstpay_phase1\firstpay_phase_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97EB5C38-A5B9-4A03-A70A-44E7F8EE7F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63F43C4-640A-4E49-BAD8-0721C0D1EAB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="965" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="965" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VP Ratings" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="38">
   <si>
     <t>Emp No</t>
   </si>
@@ -626,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.21875" style="1" bestFit="1" customWidth="1"/>
@@ -676,6 +676,76 @@
       </c>
       <c r="K1" s="15" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="1">
+        <v>3</v>
+      </c>
+      <c r="G2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H2">
+        <v>1.2</v>
+      </c>
+      <c r="I2">
+        <v>50000</v>
+      </c>
+      <c r="J2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="1">
+        <v>2</v>
+      </c>
+      <c r="G3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H3">
+        <v>1.2</v>
+      </c>
+      <c r="I3">
+        <v>123</v>
+      </c>
+      <c r="J3" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>